<commit_message>
Update Dataset function, add missing collumn to example and add missing collumn to example and to chroma db, fix rating and rag engine for higher score and source error in result.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dataset/example_sheet.xlsx
+++ b/Dataset/example_sheet.xlsx
@@ -524,6 +524,11 @@
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -536,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -547,37 +552,67 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>question_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>difficulty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>question_vi</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>expected_answer_vi</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>article_reference</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ground_truth_rule</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>question_type</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>difficulty</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>split</t>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>retrieval_keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>expected_retrieved_context</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>evaluation_focus</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
@@ -589,37 +624,67 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>công ty trách nhiệm hữu hạn một thành viên</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Công ty TNHH một thành viên là gì?</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Là doanh nghiệp do một tổ chức hoặc một cá nhân làm chủ sở hữu; chủ sở hữu chịu trách nhiệm về các khoản nợ trong phạm vi số vốn điều lệ.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Điều 4</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Công ty TNHH một thành viên do một chủ sở hữu, chịu trách nhiệm hữu hạn trong phạm vi vốn điều lệ.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>factual</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>easy</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>demo</t>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>công ty TNHH một thành viên;chủ sở hữu;trách nhiệm hữu hạn</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Điều 4. Công ty TNHH một thành viên là doanh nghiệp do một tổ chức hoặc một cá nhân làm chủ sở hữu; chủ sở hữu công ty chịu trách nhiệm về các khoản nợ và nghĩa vụ tài sản khác của công ty trong phạm vi số vốn điều lệ.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>định nghĩa loại hình doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
         </is>
       </c>
     </row>
@@ -631,37 +696,67 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>quyền thành lập doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Ai có quyền thành lập doanh nghiệp?</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Mọi tổ chức, cá nhân đều có quyền thành lập và quản lý doanh nghiệp, trừ các trường hợp bị pháp luật cấm.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Điều 17</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Quyền thành lập doanh nghiệp là quyền chung, trừ trường hợp bị cấm.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>test</t>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>quyền thành lập;điều kiện thành lập;cấm thành lập</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Điều 17. Tổ chức, cá nhân có quyền thành lập và quản lý doanh nghiệp, trừ các trường hợp bị cấm theo quy định của pháp luật.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>điều kiện/chủ thể có quyền thành lập</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
         </is>
       </c>
     </row>
@@ -676,7 +771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -687,37 +782,67 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>question_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>difficulty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>question_vi</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>expected_answer_vi</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>article_reference</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ground_truth_rule</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>question_type</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>difficulty</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>split</t>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>retrieval_keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>expected_retrieved_context</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>evaluation_focus</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
@@ -729,37 +854,67 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>factual</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>công ty trách nhiệm hữu hạn một thành viên</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Công ty TNHH một thành viên là gì?</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Là doanh nghiệp do một tổ chức hoặc một cá nhân làm chủ sở hữu; chủ sở hữu chịu trách nhiệm về các khoản nợ trong phạm vi số vốn điều lệ.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Điều 4</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Công ty TNHH một thành viên do một chủ sở hữu, chịu trách nhiệm hữu hạn trong phạm vi vốn điều lệ.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>factual</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>easy</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>demo</t>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>công ty TNHH một thành viên;chủ sở hữu;trách nhiệm hữu hạn</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Điều 4. Công ty TNHH một thành viên là doanh nghiệp do một tổ chức hoặc một cá nhân làm chủ sở hữu; chủ sở hữu công ty chịu trách nhiệm về các khoản nợ và nghĩa vụ tài sản khác của công ty trong phạm vi số vốn điều lệ.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>định nghĩa loại hình doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
         </is>
       </c>
     </row>
@@ -774,50 +929,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>article_reference</t>
+          <t>update_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>topic</t>
+          <t>date/effective</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>impact</t>
+          <t>legal_source</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>effective_date</t>
+          <t>key_change_vi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>impact_on_dataset</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>implemented_in_sheet</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Điều 17</t>
+          <t>UPD001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>mở rộng quyền thành lập doanh nghiệp</t>
+          <t>01/07/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bổ sung một số trường hợp được miễn hạn chế thành lập doanh nghiệp so với luật cũ.</t>
+          <t>Luật Doanh nghiệp 2020</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>Mở rộng quyền thành lập doanh nghiệp — bổ sung một số trường hợp được miễn hạn chế thành lập doanh nghiệp so với luật cũ.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cập nhật Điều 17 trong Dataset_example, Demo_Quick_example.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Dataset_example; Demo_Quick_example</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update fix keyword function error, fix bug in dataset, update rag engine for better chat
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dataset/example_sheet.xlsx
+++ b/Dataset/example_sheet.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KB_Articles" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,13 +20,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,13 +54,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -128,7 +134,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -171,71 +177,13 @@
     <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -243,7 +191,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -266,7 +214,7 @@
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -357,7 +305,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -379,11 +327,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
+          <a:path path="circle"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -398,15 +344,12 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:path path="circle"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -416,7 +359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,10 +390,15 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>so_ky_hieu</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -484,10 +432,15 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>59/2020/QH14</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
         </is>
@@ -521,12 +474,59 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>59/2020/QH14</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Điều 52 Nghị định 168/2025/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Thông báo thay đổi thông tin chủ sở hữu hưởng lợi</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Doanh nghiệp thông báo trong thời hạn 10 ngày khi có thay đổi thông tin chủ sở hữu hưởng lợi hoặc tỷ lệ sở hữu đã kê khai.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>thay đổi chủ sở hữu hưởng lợi;10 ngày;công ty cổ phần</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>decree=168; article=52; type=beneficial_owner_change</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>168/2025/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://xaydungchinhsach.chinhphu.vn/toan-van-nghi-dinh-168-2025-nd-cp-ve-dang-ky-doanh-nghiep-119250702175708554.htm</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>VD văn bản khác Luật Doanh nghiệp 2020 — điền đúng so_ky_hieu thực tế của văn bản</t>
         </is>
       </c>
     </row>
@@ -538,8 +538,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -761,15 +761,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -919,7 +921,9 @@
       </c>
     </row>
   </sheetData>
+  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
 </worksheet>
 </file>
 
@@ -929,7 +933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -965,10 +969,15 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>so_ky_hieu</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -1007,10 +1016,15 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>59/2020/QH14</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>https://vbpl.vn/TW/Pages/vbpq-toanvan.aspx?ItemID=147025</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Ví dụ minh hoạ — điền dữ liệu thật khi dùng</t>
         </is>

</xml_diff>